<commit_message>
Reactome-Recon lists: link PI3K binding, GYS polyglucosylation and CYP11A1 to their maps
Same processes drawn differently on the phosphoinositides, glycogen and
estrogen maps.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UEhiXyuPXhFdTBjqNiEL8p
</commit_message>
<xml_diff>
--- a/downloads/reactome-recon-lists.xlsx
+++ b/downloads/reactome-recon-lists.xlsx
@@ -6076,7 +6076,11 @@
           <t>CYP11A1 cleaves 20a,22b-DHCHOL</t>
         </is>
       </c>
-      <c r="G159" s="2" t="n"/>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>Estradiol</t>
+        </is>
+      </c>
       <c r="H159" s="2" t="n"/>
       <c r="I159" s="2" t="n"/>
     </row>
@@ -14807,7 +14811,11 @@
           <t>PI3K binds to EGF:EGFR:GRB2:GAB1</t>
         </is>
       </c>
-      <c r="G408" s="2" t="n"/>
+      <c r="G408" s="3" t="inlineStr">
+        <is>
+          <t>Inositol phosphate</t>
+        </is>
+      </c>
       <c r="H408" s="2" t="n"/>
       <c r="I408" s="2" t="n"/>
     </row>
@@ -24930,7 +24938,11 @@
           <t>GYS1 catalyzes the polyglucosylation of oligoGlc-GYG1</t>
         </is>
       </c>
-      <c r="G697" s="2" t="n"/>
+      <c r="G697" s="3" t="inlineStr">
+        <is>
+          <t>Glycogen</t>
+        </is>
+      </c>
       <c r="H697" s="2" t="n"/>
       <c r="I697" s="2" t="n"/>
     </row>
@@ -25210,7 +25222,11 @@
           <t>GYS2 catalyzes the polyglucosylation of oligoGlc-GYG2</t>
         </is>
       </c>
-      <c r="G705" s="2" t="n"/>
+      <c r="G705" s="3" t="inlineStr">
+        <is>
+          <t>Glycogen</t>
+        </is>
+      </c>
       <c r="H705" s="2" t="n"/>
       <c r="I705" s="2" t="n"/>
     </row>
@@ -30250,7 +30266,11 @@
           <t>PI3K binds to EGF:EGFR:GRB2:GAB1</t>
         </is>
       </c>
-      <c r="G849" s="2" t="n"/>
+      <c r="G849" s="3" t="inlineStr">
+        <is>
+          <t>Inositol phosphate</t>
+        </is>
+      </c>
       <c r="H849" s="2" t="n"/>
       <c r="I849" s="2" t="n"/>
     </row>
@@ -31475,7 +31495,11 @@
           <t>Binding of PIK3 regulatory alpha subunit to GRB2:GAB1</t>
         </is>
       </c>
-      <c r="G884" s="2" t="n"/>
+      <c r="G884" s="3" t="inlineStr">
+        <is>
+          <t>Inositol phosphate</t>
+        </is>
+      </c>
       <c r="H884" s="2" t="n"/>
       <c r="I884" s="2" t="n"/>
     </row>
@@ -31720,7 +31744,11 @@
           <t>PI3K binds to EGF:EGFR:GRB2:GAB1</t>
         </is>
       </c>
-      <c r="G891" s="2" t="n"/>
+      <c r="G891" s="3" t="inlineStr">
+        <is>
+          <t>Inositol phosphate</t>
+        </is>
+      </c>
       <c r="H891" s="2" t="n"/>
       <c r="I891" s="2" t="n"/>
     </row>
@@ -37797,1804 +37825,1811 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F158" r:id="rId329"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId330"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F159" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F160" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F161" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F165" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F166" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F167" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F168" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F169" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F170" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D171" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F171" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F173" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D174" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F180" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D182" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D183" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D184" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D185" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D186" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D187" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F187" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D188" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D189" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F189" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D190" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F190" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G190" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D191" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F191" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D192" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F192" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G192" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D193" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F193" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D194" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F194" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D195" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D196" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D204" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F208" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F211" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F214" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F215" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F216" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F217" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F218" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D219" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F219" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F220" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D221" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F221" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F222" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F223" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F224" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F225" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F226" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F227" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F228" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F229" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F230" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F231" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F232" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F233" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D234" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F234" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F235" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D236" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F236" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F237" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F238" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F239" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F240" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F241" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F242" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F243" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F244" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F245" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D246" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F246" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F247" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F248" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F249" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D252" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D253" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D254" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D255" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D256" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D257" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D258" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F258" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F259" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F260" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D264" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D265" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D266" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F266" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F267" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D268" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F268" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D269" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F269" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D270" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F270" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D271" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F271" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D272" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F272" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D273" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F273" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D274" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F274" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D275" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F275" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D276" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F276" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D277" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F277" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D278" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F278" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D279" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F279" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D280" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F280" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D281" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F281" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D282" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F282" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D283" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F283" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D284" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F284" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D285" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F285" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D286" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F286" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D287" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F287" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D288" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F288" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D289" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F289" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D290" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F290" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D291" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F291" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D292" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F292" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D293" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F293" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D294" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F294" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D295" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F295" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D296" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F296" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D297" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F297" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D298" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F298" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D299" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F299" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D300" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F300" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D301" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F301" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D302" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F302" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D303" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F303" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D304" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F304" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D305" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F305" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D306" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F306" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D307" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F307" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D308" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F308" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D309" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F309" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D310" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F310" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D311" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F311" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D312" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F312" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D313" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F313" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D314" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F314" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D315" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F315" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D316" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F316" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D317" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F317" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D318" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F318" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D319" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F319" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D320" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F320" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D321" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F321" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D322" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F322" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D323" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F323" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D324" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F324" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D325" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F325" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D326" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F326" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D327" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F327" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D328" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F328" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D329" r:id="rId672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F329" r:id="rId673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D330" r:id="rId674"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F330" r:id="rId675"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D331" r:id="rId676"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F331" r:id="rId677"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D332" r:id="rId678"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F332" r:id="rId679"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D333" r:id="rId680"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F333" r:id="rId681"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D334" r:id="rId682"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F334" r:id="rId683"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D335" r:id="rId684"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F335" r:id="rId685"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D336" r:id="rId686"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F336" r:id="rId687"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D337" r:id="rId688"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F337" r:id="rId689"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D338" r:id="rId690"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F338" r:id="rId691"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D339" r:id="rId692"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F339" r:id="rId693"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D340" r:id="rId694"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F340" r:id="rId695"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D341" r:id="rId696"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F341" r:id="rId697"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D342" r:id="rId698"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F342" r:id="rId699"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D343" r:id="rId700"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F343" r:id="rId701"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D344" r:id="rId702"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F344" r:id="rId703"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D345" r:id="rId704"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F345" r:id="rId705"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D346" r:id="rId706"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F346" r:id="rId707"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId708"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D347" r:id="rId709"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F347" r:id="rId710"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId711"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D348" r:id="rId712"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F348" r:id="rId713"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D349" r:id="rId714"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F349" r:id="rId715"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D350" r:id="rId716"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F350" r:id="rId717"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D351" r:id="rId718"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F351" r:id="rId719"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D352" r:id="rId720"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F352" r:id="rId721"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D353" r:id="rId722"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F353" r:id="rId723"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D354" r:id="rId724"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F354" r:id="rId725"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D355" r:id="rId726"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F355" r:id="rId727"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D356" r:id="rId728"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F356" r:id="rId729"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D357" r:id="rId730"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F357" r:id="rId731"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D358" r:id="rId732"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F358" r:id="rId733"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D359" r:id="rId734"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F359" r:id="rId735"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D360" r:id="rId736"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F360" r:id="rId737"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D361" r:id="rId738"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F361" r:id="rId739"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D362" r:id="rId740"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F362" r:id="rId741"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D363" r:id="rId742"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F363" r:id="rId743"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D364" r:id="rId744"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F364" r:id="rId745"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D365" r:id="rId746"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F365" r:id="rId747"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D366" r:id="rId748"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F366" r:id="rId749"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D367" r:id="rId750"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F367" r:id="rId751"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D368" r:id="rId752"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F368" r:id="rId753"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D369" r:id="rId754"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F369" r:id="rId755"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D370" r:id="rId756"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F370" r:id="rId757"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D371" r:id="rId758"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F371" r:id="rId759"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D372" r:id="rId760"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F372" r:id="rId761"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D373" r:id="rId762"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F373" r:id="rId763"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D374" r:id="rId764"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F374" r:id="rId765"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D375" r:id="rId766"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F375" r:id="rId767"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D376" r:id="rId768"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F376" r:id="rId769"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D377" r:id="rId770"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F377" r:id="rId771"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D378" r:id="rId772"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F378" r:id="rId773"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D379" r:id="rId774"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F379" r:id="rId775"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D380" r:id="rId776"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F380" r:id="rId777"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D381" r:id="rId778"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F381" r:id="rId779"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D382" r:id="rId780"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F382" r:id="rId781"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D383" r:id="rId782"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F383" r:id="rId783"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D384" r:id="rId784"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F384" r:id="rId785"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D385" r:id="rId786"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F385" r:id="rId787"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D386" r:id="rId788"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F386" r:id="rId789"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D387" r:id="rId790"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F387" r:id="rId791"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D388" r:id="rId792"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F388" r:id="rId793"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D389" r:id="rId794"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F389" r:id="rId795"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D390" r:id="rId796"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F390" r:id="rId797"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D391" r:id="rId798"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F391" r:id="rId799"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D392" r:id="rId800"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F392" r:id="rId801"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D393" r:id="rId802"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F393" r:id="rId803"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D394" r:id="rId804"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F394" r:id="rId805"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D395" r:id="rId806"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F395" r:id="rId807"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D396" r:id="rId808"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F396" r:id="rId809"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D397" r:id="rId810"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F397" r:id="rId811"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D398" r:id="rId812"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F398" r:id="rId813"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D399" r:id="rId814"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F399" r:id="rId815"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D400" r:id="rId816"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F400" r:id="rId817"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D401" r:id="rId818"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F401" r:id="rId819"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D402" r:id="rId820"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F402" r:id="rId821"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D403" r:id="rId822"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F403" r:id="rId823"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D404" r:id="rId824"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F404" r:id="rId825"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D405" r:id="rId826"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F405" r:id="rId827"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D406" r:id="rId828"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F406" r:id="rId829"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D407" r:id="rId830"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F407" r:id="rId831"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D408" r:id="rId832"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F408" r:id="rId833"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D409" r:id="rId834"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F409" r:id="rId835"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D410" r:id="rId836"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F410" r:id="rId837"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D411" r:id="rId838"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F411" r:id="rId839"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D412" r:id="rId840"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F412" r:id="rId841"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D413" r:id="rId842"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F413" r:id="rId843"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D414" r:id="rId844"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F414" r:id="rId845"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D415" r:id="rId846"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F415" r:id="rId847"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D416" r:id="rId848"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F416" r:id="rId849"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D417" r:id="rId850"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F417" r:id="rId851"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D418" r:id="rId852"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F418" r:id="rId853"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D419" r:id="rId854"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F419" r:id="rId855"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D420" r:id="rId856"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F420" r:id="rId857"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D421" r:id="rId858"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F421" r:id="rId859"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D422" r:id="rId860"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F422" r:id="rId861"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D423" r:id="rId862"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F423" r:id="rId863"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D424" r:id="rId864"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F424" r:id="rId865"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D425" r:id="rId866"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F425" r:id="rId867"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D426" r:id="rId868"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F426" r:id="rId869"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D427" r:id="rId870"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F427" r:id="rId871"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D428" r:id="rId872"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F428" r:id="rId873"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D429" r:id="rId874"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F429" r:id="rId875"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D430" r:id="rId876"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F430" r:id="rId877"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D431" r:id="rId878"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F431" r:id="rId879"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D432" r:id="rId880"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F432" r:id="rId881"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D433" r:id="rId882"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F433" r:id="rId883"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D434" r:id="rId884"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F434" r:id="rId885"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D435" r:id="rId886"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F435" r:id="rId887"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D436" r:id="rId888"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F436" r:id="rId889"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D437" r:id="rId890"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F437" r:id="rId891"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D438" r:id="rId892"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F438" r:id="rId893"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D439" r:id="rId894"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F439" r:id="rId895"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D440" r:id="rId896"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F440" r:id="rId897"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D441" r:id="rId898"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F441" r:id="rId899"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D442" r:id="rId900"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F442" r:id="rId901"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D443" r:id="rId902"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F443" r:id="rId903"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D444" r:id="rId904"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F444" r:id="rId905"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D445" r:id="rId906"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F445" r:id="rId907"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D446" r:id="rId908"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F446" r:id="rId909"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D447" r:id="rId910"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F447" r:id="rId911"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D448" r:id="rId912"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F448" r:id="rId913"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D449" r:id="rId914"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F449" r:id="rId915"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D450" r:id="rId916"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F450" r:id="rId917"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D451" r:id="rId918"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F451" r:id="rId919"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D452" r:id="rId920"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F452" r:id="rId921"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D453" r:id="rId922"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F453" r:id="rId923"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D454" r:id="rId924"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F454" r:id="rId925"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D455" r:id="rId926"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F455" r:id="rId927"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D456" r:id="rId928"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F456" r:id="rId929"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D457" r:id="rId930"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F457" r:id="rId931"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D458" r:id="rId932"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F458" r:id="rId933"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D459" r:id="rId934"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F459" r:id="rId935"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D460" r:id="rId936"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F460" r:id="rId937"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D461" r:id="rId938"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F461" r:id="rId939"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D462" r:id="rId940"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F462" r:id="rId941"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D463" r:id="rId942"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F463" r:id="rId943"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D464" r:id="rId944"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F464" r:id="rId945"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D465" r:id="rId946"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F465" r:id="rId947"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D466" r:id="rId948"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F466" r:id="rId949"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D467" r:id="rId950"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F467" r:id="rId951"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D468" r:id="rId952"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F468" r:id="rId953"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D469" r:id="rId954"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F469" r:id="rId955"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D470" r:id="rId956"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F470" r:id="rId957"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D471" r:id="rId958"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F471" r:id="rId959"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D472" r:id="rId960"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F472" r:id="rId961"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D473" r:id="rId962"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F473" r:id="rId963"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D474" r:id="rId964"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F474" r:id="rId965"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D475" r:id="rId966"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F475" r:id="rId967"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D476" r:id="rId968"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F476" r:id="rId969"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D477" r:id="rId970"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F477" r:id="rId971"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D478" r:id="rId972"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F478" r:id="rId973"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D479" r:id="rId974"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F479" r:id="rId975"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D480" r:id="rId976"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F480" r:id="rId977"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D481" r:id="rId978"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F481" r:id="rId979"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D482" r:id="rId980"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F482" r:id="rId981"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D483" r:id="rId982"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F483" r:id="rId983"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D484" r:id="rId984"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F484" r:id="rId985"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D485" r:id="rId986"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F485" r:id="rId987"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D486" r:id="rId988"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F486" r:id="rId989"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D487" r:id="rId990"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F487" r:id="rId991"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D488" r:id="rId992"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F488" r:id="rId993"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D489" r:id="rId994"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F489" r:id="rId995"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D490" r:id="rId996"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F490" r:id="rId997"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D491" r:id="rId998"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F491" r:id="rId999"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D492" r:id="rId1000"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F492" r:id="rId1001"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D493" r:id="rId1002"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F493" r:id="rId1003"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D494" r:id="rId1004"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F494" r:id="rId1005"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D495" r:id="rId1006"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F495" r:id="rId1007"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D496" r:id="rId1008"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F496" r:id="rId1009"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D497" r:id="rId1010"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F497" r:id="rId1011"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D498" r:id="rId1012"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F498" r:id="rId1013"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D499" r:id="rId1014"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F499" r:id="rId1015"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D500" r:id="rId1016"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F500" r:id="rId1017"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D501" r:id="rId1018"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F501" r:id="rId1019"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D502" r:id="rId1020"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F502" r:id="rId1021"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D503" r:id="rId1022"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F503" r:id="rId1023"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D504" r:id="rId1024"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F504" r:id="rId1025"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D505" r:id="rId1026"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F505" r:id="rId1027"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D506" r:id="rId1028"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F506" r:id="rId1029"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D507" r:id="rId1030"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F507" r:id="rId1031"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D508" r:id="rId1032"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F508" r:id="rId1033"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D509" r:id="rId1034"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F509" r:id="rId1035"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D510" r:id="rId1036"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F510" r:id="rId1037"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D511" r:id="rId1038"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F511" r:id="rId1039"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D512" r:id="rId1040"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F512" r:id="rId1041"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D513" r:id="rId1042"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F513" r:id="rId1043"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D514" r:id="rId1044"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F514" r:id="rId1045"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D515" r:id="rId1046"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F515" r:id="rId1047"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D516" r:id="rId1048"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F516" r:id="rId1049"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D517" r:id="rId1050"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F517" r:id="rId1051"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D518" r:id="rId1052"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F518" r:id="rId1053"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G518" r:id="rId1054"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D519" r:id="rId1055"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F519" r:id="rId1056"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D520" r:id="rId1057"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F520" r:id="rId1058"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D521" r:id="rId1059"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F521" r:id="rId1060"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G521" r:id="rId1061"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D522" r:id="rId1062"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F522" r:id="rId1063"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D523" r:id="rId1064"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F523" r:id="rId1065"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D524" r:id="rId1066"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F524" r:id="rId1067"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D525" r:id="rId1068"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F525" r:id="rId1069"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D526" r:id="rId1070"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F526" r:id="rId1071"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D527" r:id="rId1072"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F527" r:id="rId1073"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D528" r:id="rId1074"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F528" r:id="rId1075"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D529" r:id="rId1076"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F529" r:id="rId1077"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D530" r:id="rId1078"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F530" r:id="rId1079"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D531" r:id="rId1080"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F531" r:id="rId1081"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D532" r:id="rId1082"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F532" r:id="rId1083"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D533" r:id="rId1084"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F533" r:id="rId1085"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D534" r:id="rId1086"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F534" r:id="rId1087"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D535" r:id="rId1088"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F535" r:id="rId1089"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D536" r:id="rId1090"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F536" r:id="rId1091"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D537" r:id="rId1092"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F537" r:id="rId1093"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D538" r:id="rId1094"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F538" r:id="rId1095"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D539" r:id="rId1096"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F539" r:id="rId1097"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D540" r:id="rId1098"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F540" r:id="rId1099"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D541" r:id="rId1100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F541" r:id="rId1101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D542" r:id="rId1102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F542" r:id="rId1103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D543" r:id="rId1104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F543" r:id="rId1105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D544" r:id="rId1106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F544" r:id="rId1107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D545" r:id="rId1108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F545" r:id="rId1109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D546" r:id="rId1110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F546" r:id="rId1111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D547" r:id="rId1112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F547" r:id="rId1113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D548" r:id="rId1114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F548" r:id="rId1115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D549" r:id="rId1116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F549" r:id="rId1117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D550" r:id="rId1118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F550" r:id="rId1119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D551" r:id="rId1120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F551" r:id="rId1121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D552" r:id="rId1122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F552" r:id="rId1123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D553" r:id="rId1124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F553" r:id="rId1125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D554" r:id="rId1126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F554" r:id="rId1127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D555" r:id="rId1128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F555" r:id="rId1129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D556" r:id="rId1130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F556" r:id="rId1131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D557" r:id="rId1132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F557" r:id="rId1133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D558" r:id="rId1134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F558" r:id="rId1135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D559" r:id="rId1136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F559" r:id="rId1137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D560" r:id="rId1138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F560" r:id="rId1139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D561" r:id="rId1140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F561" r:id="rId1141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D562" r:id="rId1142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F562" r:id="rId1143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D563" r:id="rId1144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F563" r:id="rId1145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D564" r:id="rId1146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F564" r:id="rId1147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D565" r:id="rId1148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F565" r:id="rId1149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D566" r:id="rId1150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F566" r:id="rId1151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D567" r:id="rId1152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F567" r:id="rId1153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D568" r:id="rId1154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F568" r:id="rId1155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D569" r:id="rId1156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F569" r:id="rId1157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D570" r:id="rId1158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F570" r:id="rId1159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D571" r:id="rId1160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F571" r:id="rId1161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D572" r:id="rId1162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F572" r:id="rId1163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D573" r:id="rId1164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F573" r:id="rId1165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D574" r:id="rId1166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F574" r:id="rId1167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D575" r:id="rId1168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F575" r:id="rId1169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D576" r:id="rId1170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F576" r:id="rId1171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D577" r:id="rId1172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F577" r:id="rId1173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D578" r:id="rId1174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F578" r:id="rId1175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D579" r:id="rId1176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F579" r:id="rId1177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D580" r:id="rId1178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F580" r:id="rId1179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D581" r:id="rId1180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F581" r:id="rId1181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D582" r:id="rId1182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F582" r:id="rId1183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D583" r:id="rId1184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F583" r:id="rId1185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D584" r:id="rId1186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F584" r:id="rId1187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D585" r:id="rId1188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F585" r:id="rId1189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D586" r:id="rId1190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F586" r:id="rId1191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D587" r:id="rId1192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F587" r:id="rId1193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D588" r:id="rId1194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F588" r:id="rId1195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D589" r:id="rId1196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F589" r:id="rId1197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D590" r:id="rId1198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F590" r:id="rId1199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D591" r:id="rId1200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F591" r:id="rId1201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D592" r:id="rId1202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F592" r:id="rId1203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D593" r:id="rId1204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F593" r:id="rId1205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D594" r:id="rId1206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F594" r:id="rId1207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D595" r:id="rId1208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F595" r:id="rId1209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D596" r:id="rId1210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F596" r:id="rId1211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D597" r:id="rId1212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F597" r:id="rId1213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D598" r:id="rId1214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F598" r:id="rId1215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D599" r:id="rId1216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F599" r:id="rId1217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D600" r:id="rId1218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F600" r:id="rId1219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D601" r:id="rId1220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F601" r:id="rId1221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D602" r:id="rId1222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F602" r:id="rId1223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D603" r:id="rId1224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F603" r:id="rId1225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D604" r:id="rId1226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F604" r:id="rId1227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D605" r:id="rId1228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F605" r:id="rId1229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D606" r:id="rId1230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F606" r:id="rId1231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D607" r:id="rId1232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F607" r:id="rId1233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D608" r:id="rId1234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F608" r:id="rId1235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D609" r:id="rId1236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F609" r:id="rId1237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D610" r:id="rId1238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F610" r:id="rId1239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D611" r:id="rId1240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F611" r:id="rId1241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D612" r:id="rId1242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F612" r:id="rId1243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D613" r:id="rId1244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F613" r:id="rId1245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D614" r:id="rId1246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F614" r:id="rId1247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D615" r:id="rId1248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F615" r:id="rId1249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D616" r:id="rId1250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F616" r:id="rId1251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D617" r:id="rId1252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F617" r:id="rId1253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D618" r:id="rId1254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F618" r:id="rId1255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D619" r:id="rId1256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F619" r:id="rId1257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D620" r:id="rId1258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F620" r:id="rId1259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D621" r:id="rId1260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F621" r:id="rId1261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D622" r:id="rId1262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F622" r:id="rId1263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D623" r:id="rId1264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F623" r:id="rId1265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D624" r:id="rId1266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F624" r:id="rId1267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D625" r:id="rId1268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F625" r:id="rId1269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D626" r:id="rId1270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F626" r:id="rId1271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D627" r:id="rId1272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F627" r:id="rId1273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D628" r:id="rId1274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F628" r:id="rId1275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D629" r:id="rId1276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F629" r:id="rId1277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D630" r:id="rId1278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F630" r:id="rId1279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D631" r:id="rId1280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F631" r:id="rId1281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D632" r:id="rId1282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F632" r:id="rId1283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D633" r:id="rId1284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F633" r:id="rId1285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D634" r:id="rId1286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F634" r:id="rId1287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D635" r:id="rId1288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F635" r:id="rId1289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D636" r:id="rId1290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F636" r:id="rId1291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D637" r:id="rId1292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F637" r:id="rId1293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D638" r:id="rId1294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F638" r:id="rId1295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D639" r:id="rId1296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F639" r:id="rId1297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D640" r:id="rId1298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F640" r:id="rId1299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D641" r:id="rId1300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F641" r:id="rId1301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D642" r:id="rId1302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F642" r:id="rId1303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D643" r:id="rId1304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F643" r:id="rId1305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D644" r:id="rId1306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F644" r:id="rId1307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D645" r:id="rId1308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F645" r:id="rId1309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D646" r:id="rId1310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F646" r:id="rId1311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D647" r:id="rId1312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F647" r:id="rId1313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D648" r:id="rId1314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F648" r:id="rId1315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D649" r:id="rId1316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F649" r:id="rId1317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D650" r:id="rId1318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F650" r:id="rId1319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D651" r:id="rId1320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F651" r:id="rId1321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D652" r:id="rId1322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F652" r:id="rId1323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D653" r:id="rId1324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F653" r:id="rId1325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D654" r:id="rId1326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F654" r:id="rId1327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D655" r:id="rId1328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F655" r:id="rId1329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D656" r:id="rId1330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F656" r:id="rId1331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D657" r:id="rId1332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F657" r:id="rId1333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D658" r:id="rId1334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F658" r:id="rId1335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D659" r:id="rId1336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F659" r:id="rId1337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D660" r:id="rId1338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F660" r:id="rId1339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D661" r:id="rId1340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F661" r:id="rId1341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D662" r:id="rId1342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F662" r:id="rId1343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D663" r:id="rId1344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F663" r:id="rId1345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D664" r:id="rId1346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F664" r:id="rId1347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D665" r:id="rId1348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F665" r:id="rId1349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D666" r:id="rId1350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F666" r:id="rId1351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D667" r:id="rId1352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F667" r:id="rId1353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D668" r:id="rId1354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F668" r:id="rId1355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D669" r:id="rId1356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F669" r:id="rId1357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D670" r:id="rId1358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F670" r:id="rId1359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D671" r:id="rId1360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F671" r:id="rId1361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D672" r:id="rId1362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F672" r:id="rId1363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D673" r:id="rId1364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F673" r:id="rId1365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D674" r:id="rId1366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F674" r:id="rId1367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D675" r:id="rId1368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F675" r:id="rId1369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D676" r:id="rId1370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F676" r:id="rId1371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D677" r:id="rId1372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F677" r:id="rId1373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D678" r:id="rId1374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F678" r:id="rId1375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D679" r:id="rId1376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F679" r:id="rId1377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D680" r:id="rId1378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F680" r:id="rId1379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D681" r:id="rId1380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F681" r:id="rId1381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D682" r:id="rId1382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F682" r:id="rId1383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D683" r:id="rId1384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F683" r:id="rId1385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D684" r:id="rId1386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F684" r:id="rId1387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D685" r:id="rId1388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F685" r:id="rId1389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D686" r:id="rId1390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F686" r:id="rId1391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D687" r:id="rId1392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F687" r:id="rId1393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D688" r:id="rId1394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F688" r:id="rId1395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D689" r:id="rId1396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F689" r:id="rId1397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D690" r:id="rId1398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F690" r:id="rId1399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D691" r:id="rId1400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F691" r:id="rId1401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D692" r:id="rId1402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F692" r:id="rId1403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D693" r:id="rId1404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F693" r:id="rId1405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D694" r:id="rId1406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F694" r:id="rId1407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D695" r:id="rId1408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F695" r:id="rId1409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D696" r:id="rId1410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F696" r:id="rId1411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D697" r:id="rId1412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F697" r:id="rId1413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D698" r:id="rId1414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F698" r:id="rId1415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D699" r:id="rId1416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F699" r:id="rId1417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D700" r:id="rId1418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F700" r:id="rId1419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D701" r:id="rId1420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F701" r:id="rId1421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D702" r:id="rId1422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F702" r:id="rId1423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D703" r:id="rId1424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F703" r:id="rId1425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D704" r:id="rId1426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F704" r:id="rId1427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D705" r:id="rId1428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F705" r:id="rId1429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D706" r:id="rId1430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F706" r:id="rId1431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D707" r:id="rId1432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F707" r:id="rId1433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D708" r:id="rId1434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F708" r:id="rId1435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D709" r:id="rId1436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F709" r:id="rId1437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D710" r:id="rId1438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F710" r:id="rId1439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D711" r:id="rId1440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F711" r:id="rId1441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D712" r:id="rId1442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F712" r:id="rId1443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D713" r:id="rId1444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F713" r:id="rId1445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D714" r:id="rId1446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F714" r:id="rId1447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D715" r:id="rId1448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F715" r:id="rId1449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D716" r:id="rId1450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F716" r:id="rId1451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D717" r:id="rId1452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F717" r:id="rId1453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D718" r:id="rId1454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F718" r:id="rId1455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D719" r:id="rId1456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F719" r:id="rId1457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D720" r:id="rId1458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F720" r:id="rId1459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D721" r:id="rId1460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F721" r:id="rId1461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D722" r:id="rId1462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F722" r:id="rId1463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D723" r:id="rId1464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F723" r:id="rId1465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D724" r:id="rId1466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F724" r:id="rId1467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D725" r:id="rId1468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F725" r:id="rId1469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D726" r:id="rId1470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F726" r:id="rId1471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D727" r:id="rId1472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F727" r:id="rId1473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D728" r:id="rId1474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F728" r:id="rId1475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D729" r:id="rId1476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F729" r:id="rId1477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D730" r:id="rId1478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F730" r:id="rId1479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D731" r:id="rId1480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F731" r:id="rId1481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D732" r:id="rId1482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F732" r:id="rId1483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D733" r:id="rId1484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F733" r:id="rId1485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D734" r:id="rId1486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F734" r:id="rId1487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D735" r:id="rId1488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F735" r:id="rId1489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D736" r:id="rId1490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F736" r:id="rId1491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D737" r:id="rId1492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F737" r:id="rId1493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D738" r:id="rId1494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F738" r:id="rId1495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D739" r:id="rId1496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F739" r:id="rId1497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D740" r:id="rId1498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F740" r:id="rId1499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D741" r:id="rId1500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F741" r:id="rId1501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D742" r:id="rId1502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F742" r:id="rId1503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D743" r:id="rId1504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F743" r:id="rId1505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D744" r:id="rId1506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F744" r:id="rId1507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D745" r:id="rId1508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F745" r:id="rId1509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D746" r:id="rId1510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F746" r:id="rId1511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D747" r:id="rId1512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F747" r:id="rId1513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D748" r:id="rId1514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F748" r:id="rId1515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D749" r:id="rId1516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F749" r:id="rId1517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D750" r:id="rId1518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F750" r:id="rId1519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D751" r:id="rId1520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F751" r:id="rId1521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D752" r:id="rId1522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F752" r:id="rId1523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D753" r:id="rId1524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F753" r:id="rId1525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D754" r:id="rId1526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F754" r:id="rId1527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D755" r:id="rId1528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F755" r:id="rId1529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D756" r:id="rId1530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F756" r:id="rId1531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D757" r:id="rId1532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F757" r:id="rId1533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D758" r:id="rId1534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F758" r:id="rId1535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D759" r:id="rId1536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F759" r:id="rId1537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D760" r:id="rId1538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F760" r:id="rId1539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D761" r:id="rId1540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F761" r:id="rId1541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D762" r:id="rId1542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F762" r:id="rId1543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D763" r:id="rId1544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F763" r:id="rId1545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D764" r:id="rId1546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F764" r:id="rId1547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D765" r:id="rId1548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F765" r:id="rId1549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D766" r:id="rId1550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F766" r:id="rId1551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D767" r:id="rId1552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F767" r:id="rId1553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D768" r:id="rId1554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F768" r:id="rId1555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D769" r:id="rId1556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F769" r:id="rId1557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D770" r:id="rId1558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F770" r:id="rId1559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D771" r:id="rId1560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F771" r:id="rId1561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D772" r:id="rId1562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F772" r:id="rId1563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D773" r:id="rId1564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F773" r:id="rId1565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D774" r:id="rId1566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F774" r:id="rId1567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D775" r:id="rId1568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F775" r:id="rId1569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D776" r:id="rId1570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F776" r:id="rId1571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D777" r:id="rId1572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F777" r:id="rId1573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D778" r:id="rId1574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F778" r:id="rId1575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D779" r:id="rId1576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F779" r:id="rId1577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D780" r:id="rId1578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F780" r:id="rId1579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D781" r:id="rId1580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F781" r:id="rId1581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D782" r:id="rId1582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F782" r:id="rId1583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D783" r:id="rId1584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F783" r:id="rId1585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D784" r:id="rId1586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F784" r:id="rId1587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D785" r:id="rId1588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F785" r:id="rId1589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D786" r:id="rId1590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F786" r:id="rId1591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D787" r:id="rId1592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F787" r:id="rId1593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D788" r:id="rId1594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F788" r:id="rId1595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D789" r:id="rId1596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F789" r:id="rId1597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D790" r:id="rId1598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F790" r:id="rId1599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D791" r:id="rId1600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F791" r:id="rId1601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D792" r:id="rId1602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F792" r:id="rId1603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D793" r:id="rId1604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F793" r:id="rId1605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D794" r:id="rId1606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F794" r:id="rId1607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D795" r:id="rId1608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F795" r:id="rId1609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D796" r:id="rId1610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F796" r:id="rId1611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D797" r:id="rId1612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F797" r:id="rId1613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D798" r:id="rId1614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F798" r:id="rId1615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D799" r:id="rId1616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F799" r:id="rId1617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D800" r:id="rId1618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F800" r:id="rId1619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D801" r:id="rId1620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F801" r:id="rId1621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D802" r:id="rId1622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F802" r:id="rId1623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D803" r:id="rId1624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F803" r:id="rId1625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D804" r:id="rId1626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F804" r:id="rId1627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D805" r:id="rId1628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F805" r:id="rId1629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D806" r:id="rId1630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F806" r:id="rId1631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D807" r:id="rId1632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F807" r:id="rId1633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D808" r:id="rId1634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F808" r:id="rId1635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D809" r:id="rId1636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F809" r:id="rId1637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D810" r:id="rId1638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F810" r:id="rId1639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D811" r:id="rId1640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F811" r:id="rId1641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D812" r:id="rId1642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F812" r:id="rId1643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D813" r:id="rId1644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F813" r:id="rId1645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D814" r:id="rId1646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F814" r:id="rId1647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D815" r:id="rId1648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F815" r:id="rId1649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D816" r:id="rId1650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F816" r:id="rId1651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D817" r:id="rId1652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F817" r:id="rId1653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D818" r:id="rId1654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F818" r:id="rId1655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D819" r:id="rId1656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F819" r:id="rId1657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D820" r:id="rId1658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F820" r:id="rId1659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D821" r:id="rId1660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F821" r:id="rId1661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D822" r:id="rId1662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F822" r:id="rId1663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D823" r:id="rId1664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F823" r:id="rId1665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D824" r:id="rId1666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F824" r:id="rId1667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D825" r:id="rId1668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F825" r:id="rId1669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D826" r:id="rId1670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F826" r:id="rId1671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D827" r:id="rId1672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F827" r:id="rId1673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D828" r:id="rId1674"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F828" r:id="rId1675"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D829" r:id="rId1676"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F829" r:id="rId1677"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D830" r:id="rId1678"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F830" r:id="rId1679"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D831" r:id="rId1680"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F831" r:id="rId1681"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D832" r:id="rId1682"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F832" r:id="rId1683"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D833" r:id="rId1684"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F833" r:id="rId1685"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D834" r:id="rId1686"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F834" r:id="rId1687"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D835" r:id="rId1688"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F835" r:id="rId1689"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D836" r:id="rId1690"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F836" r:id="rId1691"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D837" r:id="rId1692"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F837" r:id="rId1693"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D838" r:id="rId1694"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F838" r:id="rId1695"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D839" r:id="rId1696"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F839" r:id="rId1697"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D840" r:id="rId1698"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F840" r:id="rId1699"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D841" r:id="rId1700"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F841" r:id="rId1701"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D842" r:id="rId1702"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F842" r:id="rId1703"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D843" r:id="rId1704"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F843" r:id="rId1705"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D844" r:id="rId1706"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F844" r:id="rId1707"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D845" r:id="rId1708"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F845" r:id="rId1709"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D846" r:id="rId1710"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F846" r:id="rId1711"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D847" r:id="rId1712"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F847" r:id="rId1713"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D848" r:id="rId1714"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F848" r:id="rId1715"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D849" r:id="rId1716"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F849" r:id="rId1717"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D850" r:id="rId1718"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F850" r:id="rId1719"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D851" r:id="rId1720"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F851" r:id="rId1721"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D852" r:id="rId1722"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F852" r:id="rId1723"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D853" r:id="rId1724"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F853" r:id="rId1725"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D854" r:id="rId1726"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F854" r:id="rId1727"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D855" r:id="rId1728"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F855" r:id="rId1729"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D856" r:id="rId1730"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F856" r:id="rId1731"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D857" r:id="rId1732"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F857" r:id="rId1733"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D858" r:id="rId1734"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F858" r:id="rId1735"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D859" r:id="rId1736"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F859" r:id="rId1737"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D860" r:id="rId1738"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F860" r:id="rId1739"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D861" r:id="rId1740"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F861" r:id="rId1741"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D862" r:id="rId1742"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F862" r:id="rId1743"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D863" r:id="rId1744"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F863" r:id="rId1745"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D864" r:id="rId1746"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F864" r:id="rId1747"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D865" r:id="rId1748"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F865" r:id="rId1749"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D866" r:id="rId1750"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F866" r:id="rId1751"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D867" r:id="rId1752"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F867" r:id="rId1753"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D868" r:id="rId1754"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F868" r:id="rId1755"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D869" r:id="rId1756"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F869" r:id="rId1757"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D870" r:id="rId1758"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F870" r:id="rId1759"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D871" r:id="rId1760"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F871" r:id="rId1761"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D872" r:id="rId1762"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F872" r:id="rId1763"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D873" r:id="rId1764"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F873" r:id="rId1765"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D874" r:id="rId1766"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F874" r:id="rId1767"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D875" r:id="rId1768"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F875" r:id="rId1769"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D876" r:id="rId1770"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F876" r:id="rId1771"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D877" r:id="rId1772"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F877" r:id="rId1773"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D878" r:id="rId1774"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F878" r:id="rId1775"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D879" r:id="rId1776"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F879" r:id="rId1777"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D880" r:id="rId1778"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F880" r:id="rId1779"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D881" r:id="rId1780"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F881" r:id="rId1781"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D882" r:id="rId1782"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F882" r:id="rId1783"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D883" r:id="rId1784"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F883" r:id="rId1785"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D884" r:id="rId1786"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F884" r:id="rId1787"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D885" r:id="rId1788"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F885" r:id="rId1789"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D886" r:id="rId1790"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F886" r:id="rId1791"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D887" r:id="rId1792"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F887" r:id="rId1793"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D888" r:id="rId1794"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F888" r:id="rId1795"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D889" r:id="rId1796"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F889" r:id="rId1797"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D890" r:id="rId1798"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F890" r:id="rId1799"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D891" r:id="rId1800"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F891" r:id="rId1801"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D892" r:id="rId1802"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F892" r:id="rId1803"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D893" r:id="rId1804"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F893" r:id="rId1805"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D894" r:id="rId1806"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F894" r:id="rId1807"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D895" r:id="rId1808"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F895" r:id="rId1809"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D896" r:id="rId1810"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F896" r:id="rId1811"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D897" r:id="rId1812"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F897" r:id="rId1813"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D898" r:id="rId1814"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F898" r:id="rId1815"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D899" r:id="rId1816"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F899" r:id="rId1817"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D900" r:id="rId1818"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F900" r:id="rId1819"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D901" r:id="rId1820"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F901" r:id="rId1821"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D902" r:id="rId1822"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F902" r:id="rId1823"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D903" r:id="rId1824"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F903" r:id="rId1825"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D904" r:id="rId1826"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F904" r:id="rId1827"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D905" r:id="rId1828"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F905" r:id="rId1829"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D906" r:id="rId1830"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F906" r:id="rId1831"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D907" r:id="rId1832"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F907" r:id="rId1833"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D908" r:id="rId1834"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F908" r:id="rId1835"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D909" r:id="rId1836"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F909" r:id="rId1837"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D910" r:id="rId1838"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F910" r:id="rId1839"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D911" r:id="rId1840"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F911" r:id="rId1841"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D912" r:id="rId1842"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F912" r:id="rId1843"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D913" r:id="rId1844"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F913" r:id="rId1845"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D914" r:id="rId1846"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F914" r:id="rId1847"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D915" r:id="rId1848"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F915" r:id="rId1849"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D916" r:id="rId1850"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F916" r:id="rId1851"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D917" r:id="rId1852"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F917" r:id="rId1853"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D918" r:id="rId1854"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F918" r:id="rId1855"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D919" r:id="rId1856"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F919" r:id="rId1857"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D920" r:id="rId1858"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F920" r:id="rId1859"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D921" r:id="rId1860"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F921" r:id="rId1861"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D922" r:id="rId1862"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F922" r:id="rId1863"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D923" r:id="rId1864"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F923" r:id="rId1865"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D924" r:id="rId1866"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F924" r:id="rId1867"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D925" r:id="rId1868"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F925" r:id="rId1869"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D926" r:id="rId1870"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F926" r:id="rId1871"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D927" r:id="rId1872"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F927" r:id="rId1873"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D928" r:id="rId1874"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F928" r:id="rId1875"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D929" r:id="rId1876"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F929" r:id="rId1877"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D930" r:id="rId1878"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F930" r:id="rId1879"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D931" r:id="rId1880"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F931" r:id="rId1881"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D932" r:id="rId1882"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F932" r:id="rId1883"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D933" r:id="rId1884"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F933" r:id="rId1885"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D934" r:id="rId1886"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F934" r:id="rId1887"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D935" r:id="rId1888"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F935" r:id="rId1889"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D936" r:id="rId1890"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F936" r:id="rId1891"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D937" r:id="rId1892"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F937" r:id="rId1893"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D938" r:id="rId1894"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F938" r:id="rId1895"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D939" r:id="rId1896"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F939" r:id="rId1897"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D940" r:id="rId1898"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F940" r:id="rId1899"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D941" r:id="rId1900"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F941" r:id="rId1901"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D942" r:id="rId1902"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F942" r:id="rId1903"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D943" r:id="rId1904"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F943" r:id="rId1905"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D944" r:id="rId1906"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F944" r:id="rId1907"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D945" r:id="rId1908"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F945" r:id="rId1909"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D946" r:id="rId1910"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F946" r:id="rId1911"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D947" r:id="rId1912"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F947" r:id="rId1913"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D948" r:id="rId1914"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F948" r:id="rId1915"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D949" r:id="rId1916"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F949" r:id="rId1917"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D950" r:id="rId1918"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F950" r:id="rId1919"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D951" r:id="rId1920"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F951" r:id="rId1921"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D952" r:id="rId1922"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F952" r:id="rId1923"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D953" r:id="rId1924"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F953" r:id="rId1925"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D954" r:id="rId1926"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F954" r:id="rId1927"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D955" r:id="rId1928"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F955" r:id="rId1929"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D956" r:id="rId1930"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F956" r:id="rId1931"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D957" r:id="rId1932"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F957" r:id="rId1933"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D958" r:id="rId1934"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F958" r:id="rId1935"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D959" r:id="rId1936"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F959" r:id="rId1937"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D960" r:id="rId1938"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F960" r:id="rId1939"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D961" r:id="rId1940"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F961" r:id="rId1941"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D962" r:id="rId1942"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F962" r:id="rId1943"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D963" r:id="rId1944"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F963" r:id="rId1945"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D964" r:id="rId1946"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F964" r:id="rId1947"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D965" r:id="rId1948"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F965" r:id="rId1949"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D966" r:id="rId1950"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F966" r:id="rId1951"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D967" r:id="rId1952"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F967" r:id="rId1953"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D968" r:id="rId1954"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F968" r:id="rId1955"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D969" r:id="rId1956"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F969" r:id="rId1957"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D970" r:id="rId1958"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F970" r:id="rId1959"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D971" r:id="rId1960"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F971" r:id="rId1961"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D972" r:id="rId1962"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F972" r:id="rId1963"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D973" r:id="rId1964"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F973" r:id="rId1965"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D974" r:id="rId1966"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F974" r:id="rId1967"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D975" r:id="rId1968"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F975" r:id="rId1969"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D976" r:id="rId1970"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F976" r:id="rId1971"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D977" r:id="rId1972"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F977" r:id="rId1973"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D978" r:id="rId1974"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F978" r:id="rId1975"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D979" r:id="rId1976"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F979" r:id="rId1977"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D980" r:id="rId1978"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F980" r:id="rId1979"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D981" r:id="rId1980"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F981" r:id="rId1981"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D982" r:id="rId1982"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F982" r:id="rId1983"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D983" r:id="rId1984"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F983" r:id="rId1985"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D984" r:id="rId1986"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F984" r:id="rId1987"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D985" r:id="rId1988"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F985" r:id="rId1989"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D986" r:id="rId1990"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F986" r:id="rId1991"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D987" r:id="rId1992"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F987" r:id="rId1993"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D988" r:id="rId1994"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F988" r:id="rId1995"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D989" r:id="rId1996"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F989" r:id="rId1997"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D990" r:id="rId1998"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F990" r:id="rId1999"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D991" r:id="rId2000"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F991" r:id="rId2001"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D992" r:id="rId2002"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F992" r:id="rId2003"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D993" r:id="rId2004"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F993" r:id="rId2005"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D994" r:id="rId2006"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F994" r:id="rId2007"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D995" r:id="rId2008"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F995" r:id="rId2009"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D996" r:id="rId2010"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F996" r:id="rId2011"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D997" r:id="rId2012"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F997" r:id="rId2013"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D998" r:id="rId2014"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F998" r:id="rId2015"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D999" r:id="rId2016"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F999" r:id="rId2017"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1000" r:id="rId2018"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1000" r:id="rId2019"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1001" r:id="rId2020"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1001" r:id="rId2021"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1002" r:id="rId2022"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1002" r:id="rId2023"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1003" r:id="rId2024"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1003" r:id="rId2025"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1004" r:id="rId2026"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1004" r:id="rId2027"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1005" r:id="rId2028"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1005" r:id="rId2029"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1006" r:id="rId2030"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1006" r:id="rId2031"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1007" r:id="rId2032"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1007" r:id="rId2033"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1008" r:id="rId2034"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1008" r:id="rId2035"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1009" r:id="rId2036"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1009" r:id="rId2037"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1010" r:id="rId2038"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1010" r:id="rId2039"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1011" r:id="rId2040"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1011" r:id="rId2041"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1012" r:id="rId2042"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1012" r:id="rId2043"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1013" r:id="rId2044"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1013" r:id="rId2045"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1014" r:id="rId2046"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1014" r:id="rId2047"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1015" r:id="rId2048"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1015" r:id="rId2049"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1016" r:id="rId2050"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1016" r:id="rId2051"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1017" r:id="rId2052"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1017" r:id="rId2053"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1018" r:id="rId2054"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1018" r:id="rId2055"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1019" r:id="rId2056"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1019" r:id="rId2057"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1020" r:id="rId2058"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1020" r:id="rId2059"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1021" r:id="rId2060"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1021" r:id="rId2061"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1022" r:id="rId2062"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1022" r:id="rId2063"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1023" r:id="rId2064"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1023" r:id="rId2065"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1024" r:id="rId2066"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1024" r:id="rId2067"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1025" r:id="rId2068"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1025" r:id="rId2069"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1026" r:id="rId2070"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1026" r:id="rId2071"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1027" r:id="rId2072"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1027" r:id="rId2073"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1028" r:id="rId2074"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1028" r:id="rId2075"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1029" r:id="rId2076"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1029" r:id="rId2077"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1030" r:id="rId2078"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1030" r:id="rId2079"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1031" r:id="rId2080"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1031" r:id="rId2081"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1032" r:id="rId2082"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1032" r:id="rId2083"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1033" r:id="rId2084"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1033" r:id="rId2085"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1034" r:id="rId2086"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1034" r:id="rId2087"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1035" r:id="rId2088"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1035" r:id="rId2089"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1036" r:id="rId2090"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1036" r:id="rId2091"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1037" r:id="rId2092"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1037" r:id="rId2093"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1038" r:id="rId2094"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1038" r:id="rId2095"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1039" r:id="rId2096"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1039" r:id="rId2097"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1040" r:id="rId2098"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1040" r:id="rId2099"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1041" r:id="rId2100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1041" r:id="rId2101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1042" r:id="rId2102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1042" r:id="rId2103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1043" r:id="rId2104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1043" r:id="rId2105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1044" r:id="rId2106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1044" r:id="rId2107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1045" r:id="rId2108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1045" r:id="rId2109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1046" r:id="rId2110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1046" r:id="rId2111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1047" r:id="rId2112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1047" r:id="rId2113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1048" r:id="rId2114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1048" r:id="rId2115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1049" r:id="rId2116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1049" r:id="rId2117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1050" r:id="rId2118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1050" r:id="rId2119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1051" r:id="rId2120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1051" r:id="rId2121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1052" r:id="rId2122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1052" r:id="rId2123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1053" r:id="rId2124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1053" r:id="rId2125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1054" r:id="rId2126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1054" r:id="rId2127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1055" r:id="rId2128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1055" r:id="rId2129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G159" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F160" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F161" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F162" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F163" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F164" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F165" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F166" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F167" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F168" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F169" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F170" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D171" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F171" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F172" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F173" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D174" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F174" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F175" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F176" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F177" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F178" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F179" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F180" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F181" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D182" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F182" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D183" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F183" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D184" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F184" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D185" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F185" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D186" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F186" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D187" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F187" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D188" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F188" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D189" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F189" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D190" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F190" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G190" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D191" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F191" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D192" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F192" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G192" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D193" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F193" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D194" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F194" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D195" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F195" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D196" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F196" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F197" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F198" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F199" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F200" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F201" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F202" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F203" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D204" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F204" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F205" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F206" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F207" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F208" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F209" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F210" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F211" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F212" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F213" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F214" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F215" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F216" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F217" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F218" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D219" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F219" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F220" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D221" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F221" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F222" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F223" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F224" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F225" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F226" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F227" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F228" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F229" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F230" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F231" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F232" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F233" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D234" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F234" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F235" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D236" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F236" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F237" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F238" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F239" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F240" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F241" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F242" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F243" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F244" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F245" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D246" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F246" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F247" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F248" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F249" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F250" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F251" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D252" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F252" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D253" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F253" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D254" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F254" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D255" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F255" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D256" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F256" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D257" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F257" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D258" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F258" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F259" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F260" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F261" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F262" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F263" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D264" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F264" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D265" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F265" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D266" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F266" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F267" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D268" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F268" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D269" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F269" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D270" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F270" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D271" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F271" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D272" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F272" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D273" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F273" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D274" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F274" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D275" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F275" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D276" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F276" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D277" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F277" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D278" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F278" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D279" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F279" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D280" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F280" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D281" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F281" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D282" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F282" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D283" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F283" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D284" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F284" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D285" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F285" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D286" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F286" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D287" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F287" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D288" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F288" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D289" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F289" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D290" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F290" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D291" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F291" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D292" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F292" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D293" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F293" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D294" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F294" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D295" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F295" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D296" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F296" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D297" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F297" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D298" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F298" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D299" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F299" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D300" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F300" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D301" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F301" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D302" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F302" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D303" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F303" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D304" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F304" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D305" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F305" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D306" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F306" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D307" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F307" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D308" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F308" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D309" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F309" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D310" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F310" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D311" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F311" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D312" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F312" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D313" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F313" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D314" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F314" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D315" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F315" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D316" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F316" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D317" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F317" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D318" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F318" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D319" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F319" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D320" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F320" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D321" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F321" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D322" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F322" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D323" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F323" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D324" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F324" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D325" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F325" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D326" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F326" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D327" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F327" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D328" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F328" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D329" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F329" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D330" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F330" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D331" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F331" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D332" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F332" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D333" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F333" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D334" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F334" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D335" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F335" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D336" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F336" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D337" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F337" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D338" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F338" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D339" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F339" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D340" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F340" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D341" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F341" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D342" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F342" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D343" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F343" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D344" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F344" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D345" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F345" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D346" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F346" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G346" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D347" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F347" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G347" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D348" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F348" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D349" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F349" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D350" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F350" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D351" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F351" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D352" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F352" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D353" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F353" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D354" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F354" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D355" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F355" r:id="rId728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D356" r:id="rId729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F356" r:id="rId730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D357" r:id="rId731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F357" r:id="rId732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D358" r:id="rId733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F358" r:id="rId734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D359" r:id="rId735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F359" r:id="rId736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D360" r:id="rId737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F360" r:id="rId738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D361" r:id="rId739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F361" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D362" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F362" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D363" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F363" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D364" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F364" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D365" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F365" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D366" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F366" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D367" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F367" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D368" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F368" r:id="rId754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D369" r:id="rId755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F369" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D370" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F370" r:id="rId758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D371" r:id="rId759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F371" r:id="rId760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D372" r:id="rId761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F372" r:id="rId762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D373" r:id="rId763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F373" r:id="rId764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D374" r:id="rId765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F374" r:id="rId766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D375" r:id="rId767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F375" r:id="rId768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D376" r:id="rId769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F376" r:id="rId770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D377" r:id="rId771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F377" r:id="rId772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D378" r:id="rId773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F378" r:id="rId774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D379" r:id="rId775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F379" r:id="rId776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D380" r:id="rId777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F380" r:id="rId778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D381" r:id="rId779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F381" r:id="rId780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D382" r:id="rId781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F382" r:id="rId782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D383" r:id="rId783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F383" r:id="rId784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D384" r:id="rId785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F384" r:id="rId786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D385" r:id="rId787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F385" r:id="rId788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D386" r:id="rId789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F386" r:id="rId790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D387" r:id="rId791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F387" r:id="rId792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D388" r:id="rId793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F388" r:id="rId794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D389" r:id="rId795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F389" r:id="rId796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D390" r:id="rId797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F390" r:id="rId798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D391" r:id="rId799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F391" r:id="rId800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D392" r:id="rId801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F392" r:id="rId802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D393" r:id="rId803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F393" r:id="rId804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D394" r:id="rId805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F394" r:id="rId806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D395" r:id="rId807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F395" r:id="rId808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D396" r:id="rId809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F396" r:id="rId810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D397" r:id="rId811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F397" r:id="rId812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D398" r:id="rId813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F398" r:id="rId814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D399" r:id="rId815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F399" r:id="rId816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D400" r:id="rId817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F400" r:id="rId818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D401" r:id="rId819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F401" r:id="rId820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D402" r:id="rId821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F402" r:id="rId822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D403" r:id="rId823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F403" r:id="rId824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D404" r:id="rId825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F404" r:id="rId826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D405" r:id="rId827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F405" r:id="rId828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D406" r:id="rId829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F406" r:id="rId830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D407" r:id="rId831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F407" r:id="rId832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D408" r:id="rId833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F408" r:id="rId834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G408" r:id="rId835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D409" r:id="rId836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F409" r:id="rId837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D410" r:id="rId838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F410" r:id="rId839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D411" r:id="rId840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F411" r:id="rId841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D412" r:id="rId842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F412" r:id="rId843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D413" r:id="rId844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F413" r:id="rId845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D414" r:id="rId846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F414" r:id="rId847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D415" r:id="rId848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F415" r:id="rId849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D416" r:id="rId850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F416" r:id="rId851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D417" r:id="rId852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F417" r:id="rId853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D418" r:id="rId854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F418" r:id="rId855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D419" r:id="rId856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F419" r:id="rId857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D420" r:id="rId858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F420" r:id="rId859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D421" r:id="rId860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F421" r:id="rId861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D422" r:id="rId862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F422" r:id="rId863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D423" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F423" r:id="rId865"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D424" r:id="rId866"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F424" r:id="rId867"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D425" r:id="rId868"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F425" r:id="rId869"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D426" r:id="rId870"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F426" r:id="rId871"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D427" r:id="rId872"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F427" r:id="rId873"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D428" r:id="rId874"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F428" r:id="rId875"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D429" r:id="rId876"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F429" r:id="rId877"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D430" r:id="rId878"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F430" r:id="rId879"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D431" r:id="rId880"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F431" r:id="rId881"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D432" r:id="rId882"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F432" r:id="rId883"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D433" r:id="rId884"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F433" r:id="rId885"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D434" r:id="rId886"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F434" r:id="rId887"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D435" r:id="rId888"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F435" r:id="rId889"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D436" r:id="rId890"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F436" r:id="rId891"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D437" r:id="rId892"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F437" r:id="rId893"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D438" r:id="rId894"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F438" r:id="rId895"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D439" r:id="rId896"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F439" r:id="rId897"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D440" r:id="rId898"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F440" r:id="rId899"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D441" r:id="rId900"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F441" r:id="rId901"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D442" r:id="rId902"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F442" r:id="rId903"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D443" r:id="rId904"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F443" r:id="rId905"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D444" r:id="rId906"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F444" r:id="rId907"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D445" r:id="rId908"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F445" r:id="rId909"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D446" r:id="rId910"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F446" r:id="rId911"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D447" r:id="rId912"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F447" r:id="rId913"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D448" r:id="rId914"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F448" r:id="rId915"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D449" r:id="rId916"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F449" r:id="rId917"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D450" r:id="rId918"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F450" r:id="rId919"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D451" r:id="rId920"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F451" r:id="rId921"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D452" r:id="rId922"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F452" r:id="rId923"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D453" r:id="rId924"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F453" r:id="rId925"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D454" r:id="rId926"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F454" r:id="rId927"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D455" r:id="rId928"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F455" r:id="rId929"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D456" r:id="rId930"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F456" r:id="rId931"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D457" r:id="rId932"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F457" r:id="rId933"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D458" r:id="rId934"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F458" r:id="rId935"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D459" r:id="rId936"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F459" r:id="rId937"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D460" r:id="rId938"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F460" r:id="rId939"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D461" r:id="rId940"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F461" r:id="rId941"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D462" r:id="rId942"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F462" r:id="rId943"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D463" r:id="rId944"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F463" r:id="rId945"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D464" r:id="rId946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F464" r:id="rId947"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D465" r:id="rId948"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F465" r:id="rId949"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D466" r:id="rId950"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F466" r:id="rId951"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D467" r:id="rId952"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F467" r:id="rId953"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D468" r:id="rId954"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F468" r:id="rId955"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D469" r:id="rId956"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F469" r:id="rId957"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D470" r:id="rId958"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F470" r:id="rId959"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D471" r:id="rId960"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F471" r:id="rId961"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D472" r:id="rId962"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F472" r:id="rId963"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D473" r:id="rId964"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F473" r:id="rId965"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D474" r:id="rId966"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F474" r:id="rId967"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D475" r:id="rId968"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F475" r:id="rId969"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D476" r:id="rId970"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F476" r:id="rId971"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D477" r:id="rId972"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F477" r:id="rId973"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D478" r:id="rId974"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F478" r:id="rId975"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D479" r:id="rId976"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F479" r:id="rId977"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D480" r:id="rId978"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F480" r:id="rId979"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D481" r:id="rId980"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F481" r:id="rId981"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D482" r:id="rId982"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F482" r:id="rId983"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D483" r:id="rId984"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F483" r:id="rId985"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D484" r:id="rId986"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F484" r:id="rId987"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D485" r:id="rId988"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F485" r:id="rId989"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D486" r:id="rId990"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F486" r:id="rId991"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D487" r:id="rId992"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F487" r:id="rId993"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D488" r:id="rId994"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F488" r:id="rId995"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D489" r:id="rId996"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F489" r:id="rId997"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D490" r:id="rId998"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F490" r:id="rId999"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D491" r:id="rId1000"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F491" r:id="rId1001"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D492" r:id="rId1002"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F492" r:id="rId1003"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D493" r:id="rId1004"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F493" r:id="rId1005"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D494" r:id="rId1006"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F494" r:id="rId1007"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D495" r:id="rId1008"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F495" r:id="rId1009"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D496" r:id="rId1010"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F496" r:id="rId1011"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D497" r:id="rId1012"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F497" r:id="rId1013"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D498" r:id="rId1014"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F498" r:id="rId1015"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D499" r:id="rId1016"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F499" r:id="rId1017"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D500" r:id="rId1018"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F500" r:id="rId1019"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D501" r:id="rId1020"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F501" r:id="rId1021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D502" r:id="rId1022"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F502" r:id="rId1023"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D503" r:id="rId1024"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F503" r:id="rId1025"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D504" r:id="rId1026"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F504" r:id="rId1027"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D505" r:id="rId1028"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F505" r:id="rId1029"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D506" r:id="rId1030"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F506" r:id="rId1031"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D507" r:id="rId1032"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F507" r:id="rId1033"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D508" r:id="rId1034"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F508" r:id="rId1035"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D509" r:id="rId1036"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F509" r:id="rId1037"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D510" r:id="rId1038"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F510" r:id="rId1039"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D511" r:id="rId1040"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F511" r:id="rId1041"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D512" r:id="rId1042"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F512" r:id="rId1043"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D513" r:id="rId1044"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F513" r:id="rId1045"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D514" r:id="rId1046"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F514" r:id="rId1047"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D515" r:id="rId1048"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F515" r:id="rId1049"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D516" r:id="rId1050"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F516" r:id="rId1051"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D517" r:id="rId1052"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F517" r:id="rId1053"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D518" r:id="rId1054"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F518" r:id="rId1055"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G518" r:id="rId1056"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D519" r:id="rId1057"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F519" r:id="rId1058"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D520" r:id="rId1059"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F520" r:id="rId1060"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D521" r:id="rId1061"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F521" r:id="rId1062"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G521" r:id="rId1063"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D522" r:id="rId1064"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F522" r:id="rId1065"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D523" r:id="rId1066"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F523" r:id="rId1067"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D524" r:id="rId1068"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F524" r:id="rId1069"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D525" r:id="rId1070"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F525" r:id="rId1071"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D526" r:id="rId1072"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F526" r:id="rId1073"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D527" r:id="rId1074"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F527" r:id="rId1075"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D528" r:id="rId1076"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F528" r:id="rId1077"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D529" r:id="rId1078"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F529" r:id="rId1079"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D530" r:id="rId1080"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F530" r:id="rId1081"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D531" r:id="rId1082"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F531" r:id="rId1083"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D532" r:id="rId1084"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F532" r:id="rId1085"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D533" r:id="rId1086"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F533" r:id="rId1087"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D534" r:id="rId1088"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F534" r:id="rId1089"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D535" r:id="rId1090"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F535" r:id="rId1091"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D536" r:id="rId1092"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F536" r:id="rId1093"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D537" r:id="rId1094"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F537" r:id="rId1095"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D538" r:id="rId1096"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F538" r:id="rId1097"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D539" r:id="rId1098"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F539" r:id="rId1099"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D540" r:id="rId1100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F540" r:id="rId1101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D541" r:id="rId1102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F541" r:id="rId1103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D542" r:id="rId1104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F542" r:id="rId1105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D543" r:id="rId1106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F543" r:id="rId1107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D544" r:id="rId1108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F544" r:id="rId1109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D545" r:id="rId1110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F545" r:id="rId1111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D546" r:id="rId1112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F546" r:id="rId1113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D547" r:id="rId1114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F547" r:id="rId1115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D548" r:id="rId1116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F548" r:id="rId1117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D549" r:id="rId1118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F549" r:id="rId1119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D550" r:id="rId1120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F550" r:id="rId1121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D551" r:id="rId1122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F551" r:id="rId1123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D552" r:id="rId1124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F552" r:id="rId1125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D553" r:id="rId1126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F553" r:id="rId1127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D554" r:id="rId1128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F554" r:id="rId1129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D555" r:id="rId1130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F555" r:id="rId1131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D556" r:id="rId1132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F556" r:id="rId1133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D557" r:id="rId1134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F557" r:id="rId1135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D558" r:id="rId1136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F558" r:id="rId1137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D559" r:id="rId1138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F559" r:id="rId1139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D560" r:id="rId1140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F560" r:id="rId1141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D561" r:id="rId1142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F561" r:id="rId1143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D562" r:id="rId1144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F562" r:id="rId1145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D563" r:id="rId1146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F563" r:id="rId1147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D564" r:id="rId1148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F564" r:id="rId1149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D565" r:id="rId1150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F565" r:id="rId1151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D566" r:id="rId1152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F566" r:id="rId1153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D567" r:id="rId1154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F567" r:id="rId1155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D568" r:id="rId1156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F568" r:id="rId1157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D569" r:id="rId1158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F569" r:id="rId1159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D570" r:id="rId1160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F570" r:id="rId1161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D571" r:id="rId1162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F571" r:id="rId1163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D572" r:id="rId1164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F572" r:id="rId1165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D573" r:id="rId1166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F573" r:id="rId1167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D574" r:id="rId1168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F574" r:id="rId1169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D575" r:id="rId1170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F575" r:id="rId1171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D576" r:id="rId1172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F576" r:id="rId1173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D577" r:id="rId1174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F577" r:id="rId1175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D578" r:id="rId1176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F578" r:id="rId1177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D579" r:id="rId1178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F579" r:id="rId1179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D580" r:id="rId1180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F580" r:id="rId1181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D581" r:id="rId1182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F581" r:id="rId1183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D582" r:id="rId1184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F582" r:id="rId1185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D583" r:id="rId1186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F583" r:id="rId1187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D584" r:id="rId1188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F584" r:id="rId1189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D585" r:id="rId1190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F585" r:id="rId1191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D586" r:id="rId1192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F586" r:id="rId1193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D587" r:id="rId1194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F587" r:id="rId1195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D588" r:id="rId1196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F588" r:id="rId1197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D589" r:id="rId1198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F589" r:id="rId1199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D590" r:id="rId1200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F590" r:id="rId1201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D591" r:id="rId1202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F591" r:id="rId1203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D592" r:id="rId1204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F592" r:id="rId1205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D593" r:id="rId1206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F593" r:id="rId1207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D594" r:id="rId1208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F594" r:id="rId1209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D595" r:id="rId1210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F595" r:id="rId1211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D596" r:id="rId1212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F596" r:id="rId1213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D597" r:id="rId1214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F597" r:id="rId1215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D598" r:id="rId1216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F598" r:id="rId1217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D599" r:id="rId1218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F599" r:id="rId1219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D600" r:id="rId1220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F600" r:id="rId1221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D601" r:id="rId1222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F601" r:id="rId1223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D602" r:id="rId1224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F602" r:id="rId1225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D603" r:id="rId1226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F603" r:id="rId1227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D604" r:id="rId1228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F604" r:id="rId1229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D605" r:id="rId1230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F605" r:id="rId1231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D606" r:id="rId1232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F606" r:id="rId1233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D607" r:id="rId1234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F607" r:id="rId1235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D608" r:id="rId1236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F608" r:id="rId1237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D609" r:id="rId1238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F609" r:id="rId1239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D610" r:id="rId1240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F610" r:id="rId1241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D611" r:id="rId1242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F611" r:id="rId1243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D612" r:id="rId1244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F612" r:id="rId1245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D613" r:id="rId1246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F613" r:id="rId1247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D614" r:id="rId1248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F614" r:id="rId1249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D615" r:id="rId1250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F615" r:id="rId1251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D616" r:id="rId1252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F616" r:id="rId1253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D617" r:id="rId1254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F617" r:id="rId1255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D618" r:id="rId1256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F618" r:id="rId1257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D619" r:id="rId1258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F619" r:id="rId1259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D620" r:id="rId1260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F620" r:id="rId1261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D621" r:id="rId1262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F621" r:id="rId1263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D622" r:id="rId1264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F622" r:id="rId1265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D623" r:id="rId1266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F623" r:id="rId1267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D624" r:id="rId1268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F624" r:id="rId1269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D625" r:id="rId1270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F625" r:id="rId1271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D626" r:id="rId1272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F626" r:id="rId1273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D627" r:id="rId1274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F627" r:id="rId1275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D628" r:id="rId1276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F628" r:id="rId1277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D629" r:id="rId1278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F629" r:id="rId1279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D630" r:id="rId1280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F630" r:id="rId1281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D631" r:id="rId1282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F631" r:id="rId1283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D632" r:id="rId1284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F632" r:id="rId1285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D633" r:id="rId1286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F633" r:id="rId1287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D634" r:id="rId1288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F634" r:id="rId1289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D635" r:id="rId1290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F635" r:id="rId1291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D636" r:id="rId1292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F636" r:id="rId1293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D637" r:id="rId1294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F637" r:id="rId1295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D638" r:id="rId1296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F638" r:id="rId1297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D639" r:id="rId1298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F639" r:id="rId1299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D640" r:id="rId1300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F640" r:id="rId1301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D641" r:id="rId1302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F641" r:id="rId1303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D642" r:id="rId1304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F642" r:id="rId1305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D643" r:id="rId1306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F643" r:id="rId1307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D644" r:id="rId1308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F644" r:id="rId1309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D645" r:id="rId1310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F645" r:id="rId1311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D646" r:id="rId1312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F646" r:id="rId1313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D647" r:id="rId1314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F647" r:id="rId1315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D648" r:id="rId1316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F648" r:id="rId1317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D649" r:id="rId1318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F649" r:id="rId1319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D650" r:id="rId1320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F650" r:id="rId1321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D651" r:id="rId1322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F651" r:id="rId1323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D652" r:id="rId1324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F652" r:id="rId1325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D653" r:id="rId1326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F653" r:id="rId1327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D654" r:id="rId1328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F654" r:id="rId1329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D655" r:id="rId1330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F655" r:id="rId1331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D656" r:id="rId1332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F656" r:id="rId1333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D657" r:id="rId1334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F657" r:id="rId1335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D658" r:id="rId1336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F658" r:id="rId1337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D659" r:id="rId1338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F659" r:id="rId1339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D660" r:id="rId1340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F660" r:id="rId1341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D661" r:id="rId1342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F661" r:id="rId1343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D662" r:id="rId1344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F662" r:id="rId1345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D663" r:id="rId1346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F663" r:id="rId1347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D664" r:id="rId1348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F664" r:id="rId1349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D665" r:id="rId1350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F665" r:id="rId1351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D666" r:id="rId1352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F666" r:id="rId1353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D667" r:id="rId1354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F667" r:id="rId1355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D668" r:id="rId1356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F668" r:id="rId1357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D669" r:id="rId1358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F669" r:id="rId1359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D670" r:id="rId1360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F670" r:id="rId1361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D671" r:id="rId1362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F671" r:id="rId1363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D672" r:id="rId1364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F672" r:id="rId1365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D673" r:id="rId1366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F673" r:id="rId1367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D674" r:id="rId1368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F674" r:id="rId1369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D675" r:id="rId1370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F675" r:id="rId1371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D676" r:id="rId1372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F676" r:id="rId1373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D677" r:id="rId1374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F677" r:id="rId1375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D678" r:id="rId1376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F678" r:id="rId1377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D679" r:id="rId1378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F679" r:id="rId1379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D680" r:id="rId1380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F680" r:id="rId1381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D681" r:id="rId1382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F681" r:id="rId1383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D682" r:id="rId1384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F682" r:id="rId1385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D683" r:id="rId1386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F683" r:id="rId1387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D684" r:id="rId1388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F684" r:id="rId1389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D685" r:id="rId1390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F685" r:id="rId1391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D686" r:id="rId1392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F686" r:id="rId1393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D687" r:id="rId1394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F687" r:id="rId1395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D688" r:id="rId1396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F688" r:id="rId1397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D689" r:id="rId1398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F689" r:id="rId1399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D690" r:id="rId1400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F690" r:id="rId1401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D691" r:id="rId1402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F691" r:id="rId1403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D692" r:id="rId1404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F692" r:id="rId1405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D693" r:id="rId1406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F693" r:id="rId1407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D694" r:id="rId1408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F694" r:id="rId1409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D695" r:id="rId1410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F695" r:id="rId1411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D696" r:id="rId1412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F696" r:id="rId1413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D697" r:id="rId1414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F697" r:id="rId1415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G697" r:id="rId1416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D698" r:id="rId1417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F698" r:id="rId1418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D699" r:id="rId1419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F699" r:id="rId1420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D700" r:id="rId1421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F700" r:id="rId1422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D701" r:id="rId1423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F701" r:id="rId1424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D702" r:id="rId1425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F702" r:id="rId1426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D703" r:id="rId1427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F703" r:id="rId1428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D704" r:id="rId1429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F704" r:id="rId1430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D705" r:id="rId1431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F705" r:id="rId1432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G705" r:id="rId1433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D706" r:id="rId1434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F706" r:id="rId1435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D707" r:id="rId1436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F707" r:id="rId1437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D708" r:id="rId1438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F708" r:id="rId1439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D709" r:id="rId1440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F709" r:id="rId1441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D710" r:id="rId1442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F710" r:id="rId1443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D711" r:id="rId1444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F711" r:id="rId1445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D712" r:id="rId1446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F712" r:id="rId1447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D713" r:id="rId1448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F713" r:id="rId1449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D714" r:id="rId1450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F714" r:id="rId1451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D715" r:id="rId1452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F715" r:id="rId1453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D716" r:id="rId1454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F716" r:id="rId1455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D717" r:id="rId1456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F717" r:id="rId1457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D718" r:id="rId1458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F718" r:id="rId1459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D719" r:id="rId1460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F719" r:id="rId1461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D720" r:id="rId1462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F720" r:id="rId1463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D721" r:id="rId1464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F721" r:id="rId1465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D722" r:id="rId1466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F722" r:id="rId1467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D723" r:id="rId1468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F723" r:id="rId1469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D724" r:id="rId1470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F724" r:id="rId1471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D725" r:id="rId1472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F725" r:id="rId1473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D726" r:id="rId1474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F726" r:id="rId1475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D727" r:id="rId1476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F727" r:id="rId1477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D728" r:id="rId1478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F728" r:id="rId1479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D729" r:id="rId1480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F729" r:id="rId1481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D730" r:id="rId1482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F730" r:id="rId1483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D731" r:id="rId1484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F731" r:id="rId1485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D732" r:id="rId1486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F732" r:id="rId1487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D733" r:id="rId1488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F733" r:id="rId1489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D734" r:id="rId1490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F734" r:id="rId1491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D735" r:id="rId1492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F735" r:id="rId1493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D736" r:id="rId1494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F736" r:id="rId1495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D737" r:id="rId1496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F737" r:id="rId1497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D738" r:id="rId1498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F738" r:id="rId1499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D739" r:id="rId1500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F739" r:id="rId1501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D740" r:id="rId1502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F740" r:id="rId1503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D741" r:id="rId1504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F741" r:id="rId1505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D742" r:id="rId1506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F742" r:id="rId1507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D743" r:id="rId1508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F743" r:id="rId1509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D744" r:id="rId1510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F744" r:id="rId1511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D745" r:id="rId1512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F745" r:id="rId1513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D746" r:id="rId1514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F746" r:id="rId1515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D747" r:id="rId1516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F747" r:id="rId1517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D748" r:id="rId1518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F748" r:id="rId1519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D749" r:id="rId1520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F749" r:id="rId1521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D750" r:id="rId1522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F750" r:id="rId1523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D751" r:id="rId1524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F751" r:id="rId1525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D752" r:id="rId1526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F752" r:id="rId1527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D753" r:id="rId1528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F753" r:id="rId1529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D754" r:id="rId1530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F754" r:id="rId1531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D755" r:id="rId1532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F755" r:id="rId1533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D756" r:id="rId1534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F756" r:id="rId1535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D757" r:id="rId1536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F757" r:id="rId1537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D758" r:id="rId1538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F758" r:id="rId1539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D759" r:id="rId1540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F759" r:id="rId1541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D760" r:id="rId1542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F760" r:id="rId1543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D761" r:id="rId1544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F761" r:id="rId1545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D762" r:id="rId1546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F762" r:id="rId1547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D763" r:id="rId1548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F763" r:id="rId1549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D764" r:id="rId1550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F764" r:id="rId1551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D765" r:id="rId1552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F765" r:id="rId1553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D766" r:id="rId1554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F766" r:id="rId1555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D767" r:id="rId1556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F767" r:id="rId1557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D768" r:id="rId1558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F768" r:id="rId1559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D769" r:id="rId1560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F769" r:id="rId1561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D770" r:id="rId1562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F770" r:id="rId1563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D771" r:id="rId1564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F771" r:id="rId1565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D772" r:id="rId1566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F772" r:id="rId1567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D773" r:id="rId1568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F773" r:id="rId1569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D774" r:id="rId1570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F774" r:id="rId1571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D775" r:id="rId1572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F775" r:id="rId1573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D776" r:id="rId1574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F776" r:id="rId1575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D777" r:id="rId1576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F777" r:id="rId1577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D778" r:id="rId1578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F778" r:id="rId1579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D779" r:id="rId1580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F779" r:id="rId1581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D780" r:id="rId1582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F780" r:id="rId1583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D781" r:id="rId1584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F781" r:id="rId1585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D782" r:id="rId1586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F782" r:id="rId1587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D783" r:id="rId1588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F783" r:id="rId1589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D784" r:id="rId1590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F784" r:id="rId1591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D785" r:id="rId1592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F785" r:id="rId1593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D786" r:id="rId1594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F786" r:id="rId1595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D787" r:id="rId1596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F787" r:id="rId1597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D788" r:id="rId1598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F788" r:id="rId1599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D789" r:id="rId1600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F789" r:id="rId1601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D790" r:id="rId1602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F790" r:id="rId1603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D791" r:id="rId1604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F791" r:id="rId1605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D792" r:id="rId1606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F792" r:id="rId1607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D793" r:id="rId1608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F793" r:id="rId1609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D794" r:id="rId1610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F794" r:id="rId1611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D795" r:id="rId1612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F795" r:id="rId1613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D796" r:id="rId1614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F796" r:id="rId1615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D797" r:id="rId1616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F797" r:id="rId1617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D798" r:id="rId1618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F798" r:id="rId1619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D799" r:id="rId1620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F799" r:id="rId1621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D800" r:id="rId1622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F800" r:id="rId1623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D801" r:id="rId1624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F801" r:id="rId1625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D802" r:id="rId1626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F802" r:id="rId1627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D803" r:id="rId1628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F803" r:id="rId1629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D804" r:id="rId1630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F804" r:id="rId1631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D805" r:id="rId1632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F805" r:id="rId1633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D806" r:id="rId1634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F806" r:id="rId1635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D807" r:id="rId1636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F807" r:id="rId1637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D808" r:id="rId1638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F808" r:id="rId1639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D809" r:id="rId1640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F809" r:id="rId1641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D810" r:id="rId1642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F810" r:id="rId1643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D811" r:id="rId1644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F811" r:id="rId1645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D812" r:id="rId1646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F812" r:id="rId1647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D813" r:id="rId1648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F813" r:id="rId1649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D814" r:id="rId1650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F814" r:id="rId1651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D815" r:id="rId1652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F815" r:id="rId1653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D816" r:id="rId1654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F816" r:id="rId1655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D817" r:id="rId1656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F817" r:id="rId1657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D818" r:id="rId1658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F818" r:id="rId1659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D819" r:id="rId1660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F819" r:id="rId1661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D820" r:id="rId1662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F820" r:id="rId1663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D821" r:id="rId1664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F821" r:id="rId1665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D822" r:id="rId1666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F822" r:id="rId1667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D823" r:id="rId1668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F823" r:id="rId1669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D824" r:id="rId1670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F824" r:id="rId1671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D825" r:id="rId1672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F825" r:id="rId1673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D826" r:id="rId1674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F826" r:id="rId1675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D827" r:id="rId1676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F827" r:id="rId1677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D828" r:id="rId1678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F828" r:id="rId1679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D829" r:id="rId1680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F829" r:id="rId1681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D830" r:id="rId1682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F830" r:id="rId1683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D831" r:id="rId1684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F831" r:id="rId1685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D832" r:id="rId1686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F832" r:id="rId1687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D833" r:id="rId1688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F833" r:id="rId1689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D834" r:id="rId1690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F834" r:id="rId1691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D835" r:id="rId1692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F835" r:id="rId1693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D836" r:id="rId1694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F836" r:id="rId1695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D837" r:id="rId1696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F837" r:id="rId1697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D838" r:id="rId1698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F838" r:id="rId1699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D839" r:id="rId1700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F839" r:id="rId1701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D840" r:id="rId1702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F840" r:id="rId1703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D841" r:id="rId1704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F841" r:id="rId1705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D842" r:id="rId1706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F842" r:id="rId1707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D843" r:id="rId1708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F843" r:id="rId1709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D844" r:id="rId1710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F844" r:id="rId1711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D845" r:id="rId1712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F845" r:id="rId1713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D846" r:id="rId1714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F846" r:id="rId1715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D847" r:id="rId1716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F847" r:id="rId1717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D848" r:id="rId1718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F848" r:id="rId1719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D849" r:id="rId1720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F849" r:id="rId1721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G849" r:id="rId1722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D850" r:id="rId1723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F850" r:id="rId1724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D851" r:id="rId1725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F851" r:id="rId1726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D852" r:id="rId1727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F852" r:id="rId1728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D853" r:id="rId1729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F853" r:id="rId1730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D854" r:id="rId1731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F854" r:id="rId1732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D855" r:id="rId1733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F855" r:id="rId1734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D856" r:id="rId1735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F856" r:id="rId1736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D857" r:id="rId1737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F857" r:id="rId1738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D858" r:id="rId1739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F858" r:id="rId1740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D859" r:id="rId1741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F859" r:id="rId1742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D860" r:id="rId1743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F860" r:id="rId1744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D861" r:id="rId1745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F861" r:id="rId1746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D862" r:id="rId1747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F862" r:id="rId1748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D863" r:id="rId1749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F863" r:id="rId1750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D864" r:id="rId1751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F864" r:id="rId1752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D865" r:id="rId1753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F865" r:id="rId1754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D866" r:id="rId1755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F866" r:id="rId1756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D867" r:id="rId1757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F867" r:id="rId1758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D868" r:id="rId1759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F868" r:id="rId1760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D869" r:id="rId1761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F869" r:id="rId1762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D870" r:id="rId1763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F870" r:id="rId1764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D871" r:id="rId1765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F871" r:id="rId1766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D872" r:id="rId1767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F872" r:id="rId1768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D873" r:id="rId1769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F873" r:id="rId1770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D874" r:id="rId1771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F874" r:id="rId1772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D875" r:id="rId1773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F875" r:id="rId1774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D876" r:id="rId1775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F876" r:id="rId1776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D877" r:id="rId1777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F877" r:id="rId1778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D878" r:id="rId1779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F878" r:id="rId1780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D879" r:id="rId1781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F879" r:id="rId1782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D880" r:id="rId1783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F880" r:id="rId1784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D881" r:id="rId1785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F881" r:id="rId1786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D882" r:id="rId1787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F882" r:id="rId1788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D883" r:id="rId1789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F883" r:id="rId1790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D884" r:id="rId1791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F884" r:id="rId1792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G884" r:id="rId1793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D885" r:id="rId1794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F885" r:id="rId1795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D886" r:id="rId1796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F886" r:id="rId1797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D887" r:id="rId1798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F887" r:id="rId1799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D888" r:id="rId1800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F888" r:id="rId1801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D889" r:id="rId1802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F889" r:id="rId1803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D890" r:id="rId1804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F890" r:id="rId1805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D891" r:id="rId1806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F891" r:id="rId1807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G891" r:id="rId1808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D892" r:id="rId1809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F892" r:id="rId1810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D893" r:id="rId1811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F893" r:id="rId1812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D894" r:id="rId1813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F894" r:id="rId1814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D895" r:id="rId1815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F895" r:id="rId1816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D896" r:id="rId1817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F896" r:id="rId1818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D897" r:id="rId1819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F897" r:id="rId1820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D898" r:id="rId1821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F898" r:id="rId1822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D899" r:id="rId1823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F899" r:id="rId1824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D900" r:id="rId1825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F900" r:id="rId1826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D901" r:id="rId1827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F901" r:id="rId1828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D902" r:id="rId1829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F902" r:id="rId1830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D903" r:id="rId1831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F903" r:id="rId1832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D904" r:id="rId1833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F904" r:id="rId1834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D905" r:id="rId1835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F905" r:id="rId1836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D906" r:id="rId1837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F906" r:id="rId1838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D907" r:id="rId1839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F907" r:id="rId1840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D908" r:id="rId1841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F908" r:id="rId1842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D909" r:id="rId1843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F909" r:id="rId1844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D910" r:id="rId1845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F910" r:id="rId1846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D911" r:id="rId1847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F911" r:id="rId1848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D912" r:id="rId1849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F912" r:id="rId1850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D913" r:id="rId1851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F913" r:id="rId1852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D914" r:id="rId1853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F914" r:id="rId1854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D915" r:id="rId1855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F915" r:id="rId1856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D916" r:id="rId1857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F916" r:id="rId1858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D917" r:id="rId1859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F917" r:id="rId1860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D918" r:id="rId1861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F918" r:id="rId1862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D919" r:id="rId1863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F919" r:id="rId1864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D920" r:id="rId1865"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F920" r:id="rId1866"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D921" r:id="rId1867"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F921" r:id="rId1868"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D922" r:id="rId1869"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F922" r:id="rId1870"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D923" r:id="rId1871"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F923" r:id="rId1872"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D924" r:id="rId1873"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F924" r:id="rId1874"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D925" r:id="rId1875"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F925" r:id="rId1876"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D926" r:id="rId1877"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F926" r:id="rId1878"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D927" r:id="rId1879"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F927" r:id="rId1880"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D928" r:id="rId1881"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F928" r:id="rId1882"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D929" r:id="rId1883"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F929" r:id="rId1884"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D930" r:id="rId1885"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F930" r:id="rId1886"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D931" r:id="rId1887"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F931" r:id="rId1888"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D932" r:id="rId1889"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F932" r:id="rId1890"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D933" r:id="rId1891"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F933" r:id="rId1892"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D934" r:id="rId1893"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F934" r:id="rId1894"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D935" r:id="rId1895"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F935" r:id="rId1896"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D936" r:id="rId1897"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F936" r:id="rId1898"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D937" r:id="rId1899"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F937" r:id="rId1900"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D938" r:id="rId1901"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F938" r:id="rId1902"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D939" r:id="rId1903"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F939" r:id="rId1904"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D940" r:id="rId1905"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F940" r:id="rId1906"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D941" r:id="rId1907"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F941" r:id="rId1908"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D942" r:id="rId1909"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F942" r:id="rId1910"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D943" r:id="rId1911"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F943" r:id="rId1912"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D944" r:id="rId1913"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F944" r:id="rId1914"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D945" r:id="rId1915"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F945" r:id="rId1916"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D946" r:id="rId1917"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F946" r:id="rId1918"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D947" r:id="rId1919"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F947" r:id="rId1920"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D948" r:id="rId1921"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F948" r:id="rId1922"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D949" r:id="rId1923"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F949" r:id="rId1924"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D950" r:id="rId1925"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F950" r:id="rId1926"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D951" r:id="rId1927"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F951" r:id="rId1928"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D952" r:id="rId1929"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F952" r:id="rId1930"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D953" r:id="rId1931"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F953" r:id="rId1932"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D954" r:id="rId1933"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F954" r:id="rId1934"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D955" r:id="rId1935"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F955" r:id="rId1936"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D956" r:id="rId1937"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F956" r:id="rId1938"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D957" r:id="rId1939"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F957" r:id="rId1940"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D958" r:id="rId1941"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F958" r:id="rId1942"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D959" r:id="rId1943"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F959" r:id="rId1944"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D960" r:id="rId1945"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F960" r:id="rId1946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D961" r:id="rId1947"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F961" r:id="rId1948"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D962" r:id="rId1949"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F962" r:id="rId1950"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D963" r:id="rId1951"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F963" r:id="rId1952"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D964" r:id="rId1953"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F964" r:id="rId1954"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D965" r:id="rId1955"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F965" r:id="rId1956"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D966" r:id="rId1957"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F966" r:id="rId1958"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D967" r:id="rId1959"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F967" r:id="rId1960"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D968" r:id="rId1961"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F968" r:id="rId1962"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D969" r:id="rId1963"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F969" r:id="rId1964"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D970" r:id="rId1965"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F970" r:id="rId1966"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D971" r:id="rId1967"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F971" r:id="rId1968"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D972" r:id="rId1969"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F972" r:id="rId1970"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D973" r:id="rId1971"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F973" r:id="rId1972"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D974" r:id="rId1973"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F974" r:id="rId1974"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D975" r:id="rId1975"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F975" r:id="rId1976"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D976" r:id="rId1977"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F976" r:id="rId1978"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D977" r:id="rId1979"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F977" r:id="rId1980"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D978" r:id="rId1981"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F978" r:id="rId1982"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D979" r:id="rId1983"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F979" r:id="rId1984"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D980" r:id="rId1985"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F980" r:id="rId1986"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D981" r:id="rId1987"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F981" r:id="rId1988"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D982" r:id="rId1989"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F982" r:id="rId1990"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D983" r:id="rId1991"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F983" r:id="rId1992"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D984" r:id="rId1993"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F984" r:id="rId1994"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D985" r:id="rId1995"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F985" r:id="rId1996"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D986" r:id="rId1997"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F986" r:id="rId1998"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D987" r:id="rId1999"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F987" r:id="rId2000"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D988" r:id="rId2001"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F988" r:id="rId2002"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D989" r:id="rId2003"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F989" r:id="rId2004"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D990" r:id="rId2005"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F990" r:id="rId2006"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D991" r:id="rId2007"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F991" r:id="rId2008"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D992" r:id="rId2009"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F992" r:id="rId2010"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D993" r:id="rId2011"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F993" r:id="rId2012"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D994" r:id="rId2013"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F994" r:id="rId2014"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D995" r:id="rId2015"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F995" r:id="rId2016"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D996" r:id="rId2017"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F996" r:id="rId2018"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D997" r:id="rId2019"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F997" r:id="rId2020"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D998" r:id="rId2021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F998" r:id="rId2022"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D999" r:id="rId2023"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F999" r:id="rId2024"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1000" r:id="rId2025"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1000" r:id="rId2026"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1001" r:id="rId2027"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1001" r:id="rId2028"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1002" r:id="rId2029"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1002" r:id="rId2030"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1003" r:id="rId2031"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1003" r:id="rId2032"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1004" r:id="rId2033"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1004" r:id="rId2034"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1005" r:id="rId2035"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1005" r:id="rId2036"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1006" r:id="rId2037"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1006" r:id="rId2038"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1007" r:id="rId2039"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1007" r:id="rId2040"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1008" r:id="rId2041"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1008" r:id="rId2042"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1009" r:id="rId2043"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1009" r:id="rId2044"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1010" r:id="rId2045"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1010" r:id="rId2046"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1011" r:id="rId2047"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1011" r:id="rId2048"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1012" r:id="rId2049"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1012" r:id="rId2050"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1013" r:id="rId2051"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1013" r:id="rId2052"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1014" r:id="rId2053"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1014" r:id="rId2054"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1015" r:id="rId2055"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1015" r:id="rId2056"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1016" r:id="rId2057"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1016" r:id="rId2058"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1017" r:id="rId2059"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1017" r:id="rId2060"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1018" r:id="rId2061"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1018" r:id="rId2062"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1019" r:id="rId2063"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1019" r:id="rId2064"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1020" r:id="rId2065"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1020" r:id="rId2066"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1021" r:id="rId2067"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1021" r:id="rId2068"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1022" r:id="rId2069"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1022" r:id="rId2070"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1023" r:id="rId2071"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1023" r:id="rId2072"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1024" r:id="rId2073"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1024" r:id="rId2074"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1025" r:id="rId2075"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1025" r:id="rId2076"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1026" r:id="rId2077"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1026" r:id="rId2078"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1027" r:id="rId2079"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1027" r:id="rId2080"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1028" r:id="rId2081"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1028" r:id="rId2082"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1029" r:id="rId2083"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1029" r:id="rId2084"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1030" r:id="rId2085"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1030" r:id="rId2086"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1031" r:id="rId2087"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1031" r:id="rId2088"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1032" r:id="rId2089"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1032" r:id="rId2090"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1033" r:id="rId2091"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1033" r:id="rId2092"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1034" r:id="rId2093"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1034" r:id="rId2094"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1035" r:id="rId2095"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1035" r:id="rId2096"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1036" r:id="rId2097"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1036" r:id="rId2098"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1037" r:id="rId2099"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1037" r:id="rId2100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1038" r:id="rId2101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1038" r:id="rId2102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1039" r:id="rId2103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1039" r:id="rId2104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1040" r:id="rId2105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1040" r:id="rId2106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1041" r:id="rId2107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1041" r:id="rId2108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1042" r:id="rId2109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1042" r:id="rId2110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1043" r:id="rId2111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1043" r:id="rId2112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1044" r:id="rId2113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1044" r:id="rId2114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1045" r:id="rId2115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1045" r:id="rId2116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1046" r:id="rId2117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1046" r:id="rId2118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1047" r:id="rId2119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1047" r:id="rId2120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1048" r:id="rId2121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1048" r:id="rId2122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1049" r:id="rId2123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1049" r:id="rId2124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1050" r:id="rId2125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1050" r:id="rId2126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1051" r:id="rId2127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1051" r:id="rId2128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1052" r:id="rId2129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1052" r:id="rId2130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1053" r:id="rId2131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1053" r:id="rId2132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1054" r:id="rId2133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1054" r:id="rId2134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1055" r:id="rId2135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F1055" r:id="rId2136"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>